<commit_message>
Make workbook dimensions, units and ladder readable
Data-sheet dimensions were raw JSON ("[]" or [["axis","member"]]); they
now read "None (consolidated total)" or "axis = member". Unit notes say
"USD millions, except ratios (x) and percentages (%)". Oracle's Excel
ladder uses the app's $0-$12B scale with value labels and a hatched
Thereafter bar. Patched in place by patch_workbook_readability.py,
which rebinds the three manifests; builders now write the same text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -4902,7 +4902,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="225" t="str">
-        <x:v>USD millions unless x or %. Fiscal year and later TTM both span twelve months and overlap.</x:v>
+        <x:v>USD millions, except ratios (x) and percentages (%). Fiscal year and later TTM both span twelve months and overlap.</x:v>
       </x:c>
       <x:c r="B3" s="241"/>
       <x:c r="C3" s="241"/>
@@ -8417,7 +8417,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P21" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q21" s="312" t="str"/>
       <x:c r="R21" s="305" t="str">
@@ -8473,7 +8473,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P22" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q22" s="312" t="str"/>
       <x:c r="R22" s="305" t="str">
@@ -8529,7 +8529,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P23" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q23" s="312" t="str"/>
       <x:c r="R23" s="305" t="str">
@@ -8585,7 +8585,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P24" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q24" s="312" t="str"/>
       <x:c r="R24" s="305" t="str">
@@ -8641,7 +8641,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P25" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q25" s="312" t="str"/>
       <x:c r="R25" s="305" t="str">
@@ -8697,7 +8697,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P26" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q26" s="312" t="str"/>
       <x:c r="R26" s="305" t="str">
@@ -8753,7 +8753,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P27" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q27" s="312" t="str"/>
       <x:c r="R27" s="305" t="str">
@@ -8809,7 +8809,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P28" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q28" s="312" t="str"/>
       <x:c r="R28" s="305" t="str">
@@ -8865,7 +8865,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P29" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q29" s="312" t="str"/>
       <x:c r="R29" s="305" t="str">
@@ -8921,7 +8921,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P30" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q30" s="312" t="str"/>
       <x:c r="R30" s="305" t="str">
@@ -8977,7 +8977,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P31" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q31" s="312" t="str"/>
       <x:c r="R31" s="305" t="str">
@@ -9033,7 +9033,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P32" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q32" s="312" t="str"/>
       <x:c r="R32" s="305" t="str">
@@ -9089,7 +9089,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P33" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q33" s="312" t="str"/>
       <x:c r="R33" s="305" t="str">
@@ -9145,7 +9145,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P34" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q34" s="312" t="str"/>
       <x:c r="R34" s="305" t="str">
@@ -9201,7 +9201,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P35" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q35" s="312" t="str"/>
       <x:c r="R35" s="305" t="str">
@@ -9257,7 +9257,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P36" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q36" s="312" t="str"/>
       <x:c r="R36" s="305" t="str">
@@ -9311,7 +9311,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P37" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q37" s="312" t="str"/>
       <x:c r="R37" s="305" t="str">
@@ -9365,7 +9365,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P38" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q38" s="312" t="str"/>
       <x:c r="R38" s="305" t="str">
@@ -9419,7 +9419,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P39" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q39" s="312" t="str"/>
       <x:c r="R39" s="305" t="str">
@@ -9473,7 +9473,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P40" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q40" s="312" t="str"/>
       <x:c r="R40" s="305" t="str">
@@ -9527,7 +9527,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P41" s="245" t="str">
-        <x:v>[["us-gaap:FairValueByFairValueHierarchyLevelAxis","us-gaap:FairValueInputsLevel3Member"]]</x:v>
+        <x:v>us-gaap:FairValueByFairValueHierarchyLevelAxis = us-gaap:FairValueInputsLevel3Member</x:v>
       </x:c>
       <x:c r="Q41" s="312" t="str"/>
       <x:c r="R41" s="305" t="str">
@@ -9581,7 +9581,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P42" s="245" t="str">
-        <x:v>[["us-gaap:FairValueByFairValueHierarchyLevelAxis","us-gaap:FairValueInputsLevel3Member"]]</x:v>
+        <x:v>us-gaap:FairValueByFairValueHierarchyLevelAxis = us-gaap:FairValueInputsLevel3Member</x:v>
       </x:c>
       <x:c r="Q42" s="312" t="str"/>
       <x:c r="R42" s="305" t="str">
@@ -9635,7 +9635,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P43" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue2026Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue2026Member</x:v>
       </x:c>
       <x:c r="Q43" s="312" t="str"/>
       <x:c r="R43" s="305" t="str">
@@ -9689,7 +9689,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P44" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue2027Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue2027Member</x:v>
       </x:c>
       <x:c r="Q44" s="312" t="str"/>
       <x:c r="R44" s="305" t="str">
@@ -9743,7 +9743,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P45" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue2028Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue2028Member</x:v>
       </x:c>
       <x:c r="Q45" s="312" t="str"/>
       <x:c r="R45" s="305" t="str">
@@ -9797,7 +9797,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P46" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue2029Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue2029Member</x:v>
       </x:c>
       <x:c r="Q46" s="312" t="str"/>
       <x:c r="R46" s="305" t="str">
@@ -9851,7 +9851,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P47" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue2030Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue2030Member</x:v>
       </x:c>
       <x:c r="Q47" s="312" t="str"/>
       <x:c r="R47" s="305" t="str">
@@ -9905,7 +9905,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P48" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue20312040Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue20312040Member</x:v>
       </x:c>
       <x:c r="Q48" s="312" t="str"/>
       <x:c r="R48" s="305" t="str">
@@ -9959,7 +9959,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P49" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue20412050Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue20412050Member</x:v>
       </x:c>
       <x:c r="Q49" s="312" t="str"/>
       <x:c r="R49" s="305" t="str">
@@ -10013,7 +10013,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P50" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue20512060Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue20512060Member</x:v>
       </x:c>
       <x:c r="Q50" s="312" t="str"/>
       <x:c r="R50" s="305" t="str">
@@ -10067,7 +10067,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P51" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentAxis","lly:NotesDue20612070Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentAxis = lly:NotesDue20612070Member</x:v>
       </x:c>
       <x:c r="Q51" s="312" t="str"/>
       <x:c r="R51" s="305" t="str">
@@ -10121,7 +10121,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P52" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q52" s="312" t="str"/>
       <x:c r="R52" s="305" t="str">
@@ -10175,7 +10175,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P53" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q53" s="312" t="str"/>
       <x:c r="R53" s="305" t="str">
@@ -10229,7 +10229,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P54" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q54" s="312" t="str"/>
       <x:c r="R54" s="305" t="str">
@@ -10283,7 +10283,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P55" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q55" s="312" t="str"/>
       <x:c r="R55" s="305" t="str">
@@ -10337,7 +10337,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P56" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentRedemptionPeriodAxis","lly:MaturityDate2026Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentRedemptionPeriodAxis = lly:MaturityDate2026Member</x:v>
       </x:c>
       <x:c r="Q56" s="312" t="str"/>
       <x:c r="R56" s="305" t="str">
@@ -10391,7 +10391,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P57" s="245" t="str">
-        <x:v>[["us-gaap:DebtInstrumentRedemptionPeriodAxis","lly:MaturityDateDecember2029Member"]]</x:v>
+        <x:v>us-gaap:DebtInstrumentRedemptionPeriodAxis = lly:MaturityDateDecember2029Member</x:v>
       </x:c>
       <x:c r="Q57" s="312" t="str"/>
       <x:c r="R57" s="305" t="str">
@@ -10437,7 +10437,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P58" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q58" s="245" t="str">
         <x:v>Of this, $10B supports commercial paper. Not cash or verified drawable credit; do not add CP capacity again. Agreement conditions and facility-by-facility June composition are Unavailable.</x:v>
@@ -10485,7 +10485,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P59" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q59" s="245" t="str">
         <x:v>Included in the $10.1B; not another source of funds.</x:v>
@@ -10533,7 +10533,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P60" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q60" s="245" t="str">
         <x:v>Payable at closing, subject to conditions. Disclosed after quarter end; closing date, completion and funding allocation are not established here.</x:v>
@@ -10581,7 +10581,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P61" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q61" s="245" t="str">
         <x:v>Payment date Unavailable. Separate from cash already paid and from contingent-consideration fair value.</x:v>
@@ -10629,7 +10629,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P62" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q62" s="245" t="str">
         <x:v>Payment date Unavailable. Do not add to paid acquisition cash or contingent-consideration fair value.</x:v>
@@ -10677,7 +10677,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P63" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q63" s="245" t="str">
         <x:v>Already paid after June. Other July cash flows are unknown; June cash less this payment is not a current cash balance.</x:v>
@@ -10725,7 +10725,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P64" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q64" s="245" t="str">
         <x:v>Includes upfront cash and potential clinical, regulatory and commercial milestones. Includes the approximately $2B paid; do not add the two amounts or infer a precise remaining cash bill.</x:v>
@@ -10773,7 +10773,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P65" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q65" s="245" t="str">
         <x:v>Expected to be paid over up to ten years. Individual capital-call dates are Unavailable.</x:v>
@@ -10821,7 +10821,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P66" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q66" s="245" t="str">
         <x:v>Payments if specified purchases are not met under executed manufacturing and supply agreements; durations generally up to eight years. Not an unconditional $10B bill. Updated June ceiling, annual payments and overlap with other spending are Unavailable.</x:v>
@@ -10869,7 +10869,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P67" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q67" s="245" t="str">
         <x:v>Release says committed an additional $4.5B. Contractual payment schedule, spending to date and overlap with capex or supply commitments are not established by this release. Not added to debt or the $10B ceiling.</x:v>
@@ -10927,7 +10927,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P68" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q68" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -10985,7 +10985,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P69" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q69" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11043,7 +11043,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P70" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q70" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11101,7 +11101,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P71" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q71" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11159,7 +11159,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P72" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q72" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11217,7 +11217,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P73" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q73" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11275,7 +11275,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P74" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q74" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11333,7 +11333,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P75" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q75" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11391,7 +11391,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P76" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q76" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions</x:v>
@@ -11449,7 +11449,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P77" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q77" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11507,7 +11507,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P78" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q78" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11565,7 +11565,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P79" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q79" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11623,7 +11623,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P80" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q80" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11681,7 +11681,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P81" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q81" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11739,7 +11739,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P82" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q82" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11797,7 +11797,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P83" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q83" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11855,7 +11855,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P84" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q84" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -11913,7 +11913,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P85" s="245" t="str">
-        <x:v>[["us-gaap:StatementBusinessSegmentsAxis","lly:ReportableSegmentMember"]]</x:v>
+        <x:v>us-gaap:StatementBusinessSegmentsAxis = lly:ReportableSegmentMember</x:v>
       </x:c>
       <x:c r="Q85" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; exact single-segment dimension</x:v>
@@ -11971,7 +11971,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P86" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q86" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -12029,7 +12029,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P87" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q87" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -12087,7 +12087,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P88" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q88" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -12145,7 +12145,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P89" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q89" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -12203,7 +12203,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P90" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q90" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -12261,7 +12261,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P91" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q91" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -12319,7 +12319,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P92" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q92" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -12377,7 +12377,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P93" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q93" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; no dimensions; consolidated operations table only</x:v>
@@ -12435,7 +12435,7 @@
         <x:v>Inline XBRL</x:v>
       </x:c>
       <x:c r="P94" s="245" t="str">
-        <x:v>[["us-gaap:StatementBusinessSegmentsAxis","lly:ReportableSegmentMember"]]</x:v>
+        <x:v>us-gaap:StatementBusinessSegmentsAxis = lly:ReportableSegmentMember</x:v>
       </x:c>
       <x:c r="Q94" s="245" t="str">
         <x:v>Exact tag, duration, USD and Lilly CIK; exact single-segment dimension</x:v>
@@ -12483,7 +12483,7 @@
         <x:v>Reviewed contract text</x:v>
       </x:c>
       <x:c r="P95" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q95" s="245" t="str">
         <x:v>Initial issue principal, not June outstanding balance. Issued 2026-05-20. Stated maturity subject to applicable business-day, redemption and default provisions. Not added to June debt or the December carrying-amount table.</x:v>
@@ -12533,7 +12533,7 @@
         <x:v>Reviewed contract text</x:v>
       </x:c>
       <x:c r="P96" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q96" s="245" t="str">
         <x:v>Initial issue principal, not June outstanding balance. Issued 2026-05-20. Stated maturity subject to applicable business-day, redemption and default provisions. Not added to June debt or the December carrying-amount table.</x:v>
@@ -12583,7 +12583,7 @@
         <x:v>Reviewed contract text</x:v>
       </x:c>
       <x:c r="P97" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q97" s="245" t="str">
         <x:v>Initial issue principal, not June outstanding balance. Issued 2026-05-20. Stated maturity subject to applicable business-day, redemption and default provisions. Not added to June debt or the December carrying-amount table.</x:v>
@@ -12633,7 +12633,7 @@
         <x:v>Reviewed contract text</x:v>
       </x:c>
       <x:c r="P98" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q98" s="245" t="str">
         <x:v>Initial issue principal, not June outstanding balance. Issued 2026-05-20. Stated maturity subject to applicable business-day, redemption and default provisions. Not added to June debt or the December carrying-amount table.</x:v>
@@ -12683,7 +12683,7 @@
         <x:v>Reviewed contract text</x:v>
       </x:c>
       <x:c r="P99" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q99" s="245" t="str">
         <x:v>Initial issue principal, not June outstanding balance. Issued 2026-05-20. Stated maturity subject to applicable business-day, redemption and default provisions. Not added to June debt or the December carrying-amount table.</x:v>
@@ -12733,7 +12733,7 @@
         <x:v>Reviewed contract text</x:v>
       </x:c>
       <x:c r="P100" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q100" s="245" t="str">
         <x:v>Initial issue principal, not June outstanding balance. Issued 2026-05-20. Stated maturity subject to applicable business-day, redemption and default provisions. Not added to June debt or the December carrying-amount table.</x:v>
@@ -12783,7 +12783,7 @@
         <x:v>Reviewed contract text</x:v>
       </x:c>
       <x:c r="P101" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q101" s="245" t="str">
         <x:v>Initial issue principal, not June outstanding balance. Issued 2026-05-20. Stated maturity subject to applicable business-day, redemption and default provisions. Not added to June debt or the December carrying-amount table.</x:v>
@@ -12833,7 +12833,7 @@
         <x:v>Reviewed contract text</x:v>
       </x:c>
       <x:c r="P102" s="245" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q102" s="245" t="str">
         <x:v>Initial issue principal, not June outstanding balance. Issued 2026-05-20. Stated maturity subject to applicable business-day, redemption and default provisions. Not added to June debt or the December carrying-amount table.</x:v>
@@ -12883,7 +12883,7 @@
         <x:v>Reviewed filing text</x:v>
       </x:c>
       <x:c r="P103" s="263" t="str">
-        <x:v>[]</x:v>
+        <x:v>None (consolidated total)</x:v>
       </x:c>
       <x:c r="Q103" s="263" t="str">
         <x:v>Initial issue principal, not net cash proceeds, current outstanding debt or unused financing.</x:v>

</xml_diff>

<commit_message>
Add five-year balance and cash-flow charts
Each review and company workbook now charts the five checked fiscal years:
fiscal-year-end cash and baseline borrowing, and annual OCF, capital
spending (a use, below zero) and FCF. Both use annual_history_view's
checked rows; annual periods stay separate from the TTM, notes are kept,
negatives keep their sign and a missing value is a gap, never zero.

Excel charts are native, added by an XML patch (the .mjs --charts path
needs Node and the Artifact Tool runtime and would chart a gap as zero).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/lly_liquidity.xlsx
+++ b/samples/lly_liquidity.xlsx
@@ -12057,6 +12057,674 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="1">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1">
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Fiscal-year-end cash and baseline borrowing (USD millions)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Annual history'!$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Cash and equivalents</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="3987E5"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Annual history'!$B$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>FY2021</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>FY2022</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>FY2023</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>FY2024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>FY2025</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Annual history'!$B$6:$F$6</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0,,;(#,##0,,)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>3818500000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2067000000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2818600000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3268400000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7268000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Annual history'!$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Baseline borrowing</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="D95926"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Annual history'!$B$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>FY2021</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>FY2022</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>FY2023</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>FY2024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>FY2025</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Annual history'!$B$7:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0,,;(#,##0,,)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>16884700000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>16238600000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>25225300000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>33644200000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>42503000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="80"/>
+        <c:axId val="5001"/>
+        <c:axId val="5002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="5001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:latin typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="5002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="5002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000">
+                    <a:latin typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>USD millions</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0,,;(#,##0,,)" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:latin typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="5001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" b="0">
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="1000" b="0">
+          <a:latin typeface="Arial"/>
+          <a:cs typeface="Arial"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="1">
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1">
+                <a:latin typeface="Arial"/>
+              </a:rPr>
+              <a:t>Annual operating cash flow, capital spending (a use, below zero) and FCF (USD millions)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Annual history'!$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operating cash flow</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="3987E5"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Annual history'!$B$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>FY2021</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>FY2022</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>FY2023</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>FY2024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>FY2025</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Annual history'!$B$8:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0,,;(#,##0,,)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>7365900000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7585700000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4240100000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8817900000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>16813000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Annual history'!$A$61</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Capital spending (a use of cash)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7F838C"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Annual history'!$B$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>FY2021</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>FY2022</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>FY2023</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>FY2024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>FY2025</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Annual history'!$B$61:$F$61</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0,,;(#,##0,,)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>-1309800000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-1854300000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-3447600000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-5057800000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-7841000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Annual history'!$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Free cash flow</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="47627F"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Annual history'!$B$5:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>FY2021</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>FY2022</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>FY2023</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>FY2024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>FY2025</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Annual history'!$B$10:$F$10</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0,,;(#,##0,,)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>6056100000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5731400000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>792500000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3760100000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8972000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="80"/>
+        <c:axId val="5001"/>
+        <c:axId val="5002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="5001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:latin typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="5002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="5002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="D9D9D9"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000">
+                    <a:latin typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>USD millions</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0,,;(#,##0,,)" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:latin typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="5001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" b="0">
+              <a:latin typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="1000" b="0">
+          <a:latin typeface="Arial"/>
+          <a:cs typeface="Arial"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -12149,6 +12817,71 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6b2c78017318491a"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Annual chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rIdAnnualBalances"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Annual chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rIdAnnualFlows"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -23978,7 +24711,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
@@ -24297,7 +25030,38 @@
       <x:c r="F22" s="728"/>
     </x:row>
     <x:row r="23" ht="21" customHeight="1"/>
+    <x:row r="60">
+      <x:c r="A60" s="728" t="str">
+        <x:v>Chart data: capital spending as a use of cash, the negative of row 9 (missing years stay #N/A, so they leave a gap).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="749" t="str">
+        <x:v>Capital spending (a use of cash)</x:v>
+      </x:c>
+      <x:c r="B61" s="1449" t="n">
+        <x:f>IF(ISNUMBER(B9),-B9,NA())</x:f>
+        <x:v>-1309800000</x:v>
+      </x:c>
+      <x:c r="C61" s="1449" t="n">
+        <x:f>IF(ISNUMBER(C9),-C9,NA())</x:f>
+        <x:v>-1854300000</x:v>
+      </x:c>
+      <x:c r="D61" s="1449" t="n">
+        <x:f>IF(ISNUMBER(D9),-D9,NA())</x:f>
+        <x:v>-3447600000</x:v>
+      </x:c>
+      <x:c r="E61" s="1449" t="n">
+        <x:f>IF(ISNUMBER(E9),-E9,NA())</x:f>
+        <x:v>-5057800000</x:v>
+      </x:c>
+      <x:c r="F61" s="1450" t="n">
+        <x:f>IF(ISNUMBER(F9),-F9,NA())</x:f>
+        <x:v>-7841000000</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing r:id="rIdAnnualCharts"/>
 </x:worksheet>
 </file>
</xml_diff>